<commit_message>
Added a page where you can see the peppers that are in the db.
</commit_message>
<xml_diff>
--- a/pepper_list.xlsx
+++ b/pepper_list.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="59">
   <si>
     <t>name</t>
   </si>
@@ -112,79 +112,82 @@
     <t>Very hot habanero-type pepper with citrusy flavor</t>
   </si>
   <si>
+    <t>devils_tongue.jpg</t>
+  </si>
+  <si>
+    <t>USA/Caribbean</t>
+  </si>
+  <si>
+    <t>Yellow/Orange</t>
+  </si>
+  <si>
+    <t>Aji Fantasy</t>
+  </si>
+  <si>
+    <t>Mild sweet pepper with citrus notes and low heat</t>
+  </si>
+  <si>
+    <t>aji_fantasy.jpeg</t>
+  </si>
+  <si>
+    <t>South America (Peru)</t>
+  </si>
+  <si>
+    <t>Yellow</t>
+  </si>
+  <si>
+    <t>Cherry Bomb Orange</t>
+  </si>
+  <si>
+    <t>Mild to medium pepper with thick flesh and slightly sweet flavor</t>
+  </si>
+  <si>
+    <t>cherry_bomb_orange.jpg</t>
+  </si>
+  <si>
+    <t>Hungary</t>
+  </si>
+  <si>
+    <t>Orange</t>
+  </si>
+  <si>
+    <t>Naga</t>
+  </si>
+  <si>
+    <t>Extremely hot pepper related to ghost peppers</t>
+  </si>
+  <si>
+    <t>naga.jpg</t>
+  </si>
+  <si>
+    <t>India/Bangladesh</t>
+  </si>
+  <si>
+    <t>Long Horn</t>
+  </si>
+  <si>
+    <t>Long cayenne-type pepper used dried or fresh</t>
+  </si>
+  <si>
+    <t>long_horn.jpeg</t>
+  </si>
+  <si>
+    <t>Asia</t>
+  </si>
+  <si>
+    <t>Datil</t>
+  </si>
+  <si>
+    <t>Hot sweet pepper widely grown in Florida with fruity taste</t>
+  </si>
+  <si>
+    <t>datil.jpeg</t>
+  </si>
+  <si>
+    <t>USA (Florida)</t>
+  </si>
+  <si>
     <t>devil’s_tongue.jpg</t>
-  </si>
-  <si>
-    <t>USA/Caribbean</t>
-  </si>
-  <si>
-    <t>Yellow/Orange</t>
-  </si>
-  <si>
-    <t>Aji Fantasy</t>
-  </si>
-  <si>
-    <t>Mild sweet pepper with citrus notes and low heat</t>
-  </si>
-  <si>
-    <t>aji_fantasy.jpeg</t>
-  </si>
-  <si>
-    <t>South America (Peru)</t>
-  </si>
-  <si>
-    <t>Yellow</t>
-  </si>
-  <si>
-    <t>Cherry Bomb Orange</t>
-  </si>
-  <si>
-    <t>Mild to medium pepper with thick flesh and slightly sweet flavor</t>
-  </si>
-  <si>
-    <t>cherry_bomb_orange.jpg</t>
-  </si>
-  <si>
-    <t>Hungary</t>
-  </si>
-  <si>
-    <t>Orange</t>
-  </si>
-  <si>
-    <t>Naga</t>
-  </si>
-  <si>
-    <t>Extremely hot pepper related to ghost peppers</t>
-  </si>
-  <si>
-    <t>naga.jpg</t>
-  </si>
-  <si>
-    <t>India/Bangladesh</t>
-  </si>
-  <si>
-    <t>Long Horn</t>
-  </si>
-  <si>
-    <t>Long cayenne-type pepper used dried or fresh</t>
-  </si>
-  <si>
-    <t>long_horn.jpeg</t>
-  </si>
-  <si>
-    <t>Asia</t>
-  </si>
-  <si>
-    <t>Datil</t>
-  </si>
-  <si>
-    <t>Hot sweet pepper widely grown in Florida with fruity taste</t>
-  </si>
-  <si>
-    <t>datil.jpeg</t>
-  </si>
-  <si>
-    <t>USA (Florida)</t>
   </si>
 </sst>
 </file>
@@ -1968,7 +1971,7 @@
         <v>32</v>
       </c>
       <c r="C16" t="s" s="11">
-        <v>33</v>
+        <v>58</v>
       </c>
       <c r="D16" s="12">
         <v>125000</v>

</xml_diff>